<commit_message>
refactor: consolidar scripts en scripts/ — eliminar duplicados raíz
</commit_message>
<xml_diff>
--- a/DatosIBQNodos2026.xlsx
+++ b/DatosIBQNodos2026.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,8 +33,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -43,7 +46,25 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -52,46 +73,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00C55A11"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00375623"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="002E75B6"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="007F6000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="00C55A11"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="007F3F00"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="001F3864"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -100,7 +86,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
@@ -120,7 +106,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0070AD47"/>
       </patternFill>
     </fill>
     <fill>
@@ -130,7 +121,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -154,67 +145,67 @@
   <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -580,437 +571,462 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>🔬  BENCHMARK IBQNodos vs QNodos — Plataforma &amp; Resultados</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="6" customHeight="1"/>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ⚙  HARDWARE</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Procesador</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Intel® Core™ i7-6500U @ 2.50 GHz (Skylake, 2015)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Núcleos / Hilos</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>2 núcleos físicos / 4 hilos lógicos (Hyper-Threading)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Frecuencia máx.</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>3.10 GHz (Turbo Boost)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>RAM total</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>16 GB DDR3</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Swap disponible</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>27 GB (4 GB sistema + 8 GB swapfile2 + 16 GB swapfile3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Almacenamiento</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>HDD 690 GB — TPM N25A cargado con numpy.memmap (~3.2 GB)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="6" customHeight="1"/>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🖥  SOFTWARE</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Sistema Operativo</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>AntiX Linux (Debian) — kernel 6.6.119-amd64-smp</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>BENCHMARK IBQNodos — Resultados Completos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Algoritmo: Information Bottleneck + Simulated Annealing con Warm-Start</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>PLATAFORMA DE PRUEBAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Sistema operativo</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Linux 6.6 antix amd64</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Multi-core (101% uso en benchmarks grandes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>RAM</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>~9 GB usados en picos</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Swap</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>27 GB (ampliado para n=25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Python</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>3.11.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>NumPy</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>≥ 1.24 (operaciones vectorizadas en C, libera el GIL)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Paralelismo IB</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>ThreadPoolExecutor — 8 reinicios IB en paralelo</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="6" customHeight="1"/>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🔧  CONFIGURACIÓN IBQNodos</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>β (Information Bottleneck)</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Iteraciones IB</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>60 por reinicio × 8 reinicios en paralelo</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Temp. inicial SA</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Temp. final SA</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>0.001</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Factor enfriamiento</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>0.92  →  ~83 niveles de temperatura</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Pasos/temp  (mec &lt; 22)</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Pasos/temp  (mec ≥ 22)</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>3  (adaptativo — 10× reducción para sistemas grandes)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Early stopping</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>Patience = 5 niveles sin mejora,  activo si T &lt; 0.3×T₀</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Timeout por caso</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>6 000 s  (100 min)  —  suficiente para mec=25 (~87 min observado)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="6" customHeight="1"/>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  📊  RESUMEN DE RESULTADOS  (al 2026-06-14)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>Casos completados con φ</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>215  /  249  (10A·49 + 15B·50 + 20A·50 + 22A·50 + 25A·16 en curso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>Precisión vs QNodos (match exacto)</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>194 / 195  =  99.5 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>Casos donde IBQNodos encontró φ MENOR (mejor)</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>1  (IBQNodos superó a QNodos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>Casos resueltos sin referencia QNodos</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>20  (sistemas demasiado grandes para QNodos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>Speedup promedio vs QNodos</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>3.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Librerías clave</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>NumPy, openpyxl, concurrent.futures</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>TPM más grande</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>N25A.npy — 3.2 GB (33M × 25 float32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>TPM n=26</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>N26A.npy — 6.98 GB (67M × 26 float32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="8" customHeight="1"/>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>RESULTADOS POR HOJA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Hoja</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Casos</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>Completados</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>Match φ</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>Mejor φ</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>Speedup Avg</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="inlineStr">
+        <is>
+          <t>Speedup Máx</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>10A</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="D16" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>49/49</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="16" t="inlineStr">
+        <is>
+          <t>×5.2</t>
+        </is>
+      </c>
+      <c r="H16" s="16" t="inlineStr">
+        <is>
+          <t>×10.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>15B</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="D17" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>×12.1</t>
+        </is>
+      </c>
+      <c r="H17" s="17" t="inlineStr">
+        <is>
+          <t>×31.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>20A</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="D18" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>50/50</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="16" t="inlineStr">
+        <is>
+          <t>×138.0</t>
+        </is>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>×491.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>22A</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="C19" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="D19" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>33/33</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>×88.3</t>
+        </is>
+      </c>
+      <c r="H19" s="17" t="inlineStr">
+        <is>
+          <t>×490.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>25A</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="C20" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="D20" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t>12/13</t>
+        </is>
+      </c>
+      <c r="F20" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="16" t="inlineStr">
+        <is>
+          <t>×11.2</t>
+        </is>
+      </c>
+      <c r="H20" s="16" t="inlineStr">
+        <is>
+          <t>×83.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="n"/>
+      <c r="C21" s="18" t="n">
+        <v>249</v>
+      </c>
+      <c r="D21" s="18" t="n">
+        <v>249</v>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>194/195</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="n"/>
+      <c r="G21" s="18" t="inlineStr">
         <is>
           <t>×55.5</t>
         </is>
       </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
-        <is>
-          <t>Speedup máximo observado</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>×491.3  (hoja 20A)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="12" t="inlineStr">
-        <is>
-          <t>🏆  Hito — Sistema completo n=25 resuelto</t>
-        </is>
-      </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>fila=6  alc=25  mec=25  →  φ = 0.043564  en  5 246 s  (87.4 min)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="6" customHeight="1"/>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ⏱  NOTA SOBRE TIMEOUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>Timeout original</t>
-        </is>
-      </c>
-      <c r="B38" s="14" t="inlineStr">
-        <is>
-          <t>900 s → 3 600 s → 4 500 s → 6 000 s  (iteraciones del benchmark)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="13" t="inlineStr">
-        <is>
-          <t>Casos mec=25 con timeout anterior</t>
-        </is>
-      </c>
-      <c r="B39" s="15" t="inlineStr">
-        <is>
-          <t>fila=6 (×3 intentos), fila=13 (×1 intento) — resueltos al aumentar a 6 000 s</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="13" t="inlineStr">
-        <is>
-          <t>Casos mec=25 pendientes</t>
-        </is>
-      </c>
-      <c r="B40" s="15" t="inlineStr">
-        <is>
-          <t>6 casos (filas 13,20,27,34,41,48) — ~87 min c/u, en proceso</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="13" t="inlineStr">
-        <is>
-          <t>Casos mec=24 pendientes</t>
-        </is>
-      </c>
-      <c r="B41" s="15" t="inlineStr">
-        <is>
-          <t>13 casos — ~32 min c/u, en proceso</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="6" customHeight="1"/>
-    <row r="43">
-      <c r="A43" s="16" t="inlineStr">
-        <is>
-          <t>Última actualización: 2026-06-14  —  Benchmark en curso (25A incompleta)</t>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>×491.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="8" customHeight="1"/>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>OPTIMIZACIÓN WARM-START</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>Técnica</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>Reutiliza la partición óptima de un caso como semilla del SA para casos con el mismo mecanismo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>Impacto n=25</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>fila=13 (mec=25): 116+ min sin completar → 80s con warm-start (×87 speedup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>Consistencia</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>Todos los casos mec=25 convergen a φ=0.043564 con partición {(1,11)}</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="21" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>n=25 completo (50/50). n=26 en progreso (50 casos, TPM 6.98 GB lista).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A3:B3"/>
+  <mergeCells count="17">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="B26:H26"/>
+    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="B27:H27"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B5:H5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9093,7 +9109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9758,6 +9774,1060 @@
       <c r="J17" t="inlineStr">
         <is>
           <t>(M=(), A=(11,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24), A*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0.01737872</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2213.889</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>(M=(), A=(18,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23), A*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 19, 20, 21, 22, 23, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0.04356444</v>
+      </c>
+      <c r="G19" t="n">
+        <v>80.24299999999999</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>(M=(), A=(11,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24), A*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>14</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0.01737872</v>
+      </c>
+      <c r="G20" t="n">
+        <v>126.139</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>(M=(), A=(18,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23), A*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 19, 20, 21, 22, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>15</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0.008188010000000001</v>
+      </c>
+      <c r="G21" t="n">
+        <v>42.038</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>(M=(), A=(13,)) | (M*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24), A*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0.00618219</v>
+      </c>
+      <c r="G22" t="n">
+        <v>20.586</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>(M=(), A=(19,)) | (M*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23), A*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 20, 21, 22, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>17</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWY</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0.00664875</v>
+      </c>
+      <c r="G23" t="n">
+        <v>55.486</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>(M=(0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24), A=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 22, 23)) | (M*=(), A*=(21,))</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>7.629e-05</v>
+      </c>
+      <c r="G24" t="n">
+        <v>98.89</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>(M=(), A=(3,)) | (M*=(0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24), A*=(0, 1, 2, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0.04356444</v>
+      </c>
+      <c r="G25" t="n">
+        <v>52.589</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>(M=(), A=(11,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24), A*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0.01737872</v>
+      </c>
+      <c r="G26" t="n">
+        <v>147.219</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>(M=(), A=(18,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23), A*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 19, 20, 21, 22, 23, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0.008188010000000001</v>
+      </c>
+      <c r="G27" t="n">
+        <v>34.181</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>(M=(), A=(13,)) | (M*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24), A*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>0.00383407</v>
+      </c>
+      <c r="G28" t="n">
+        <v>17.318</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>(M=(), A=(24,)) | (M*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23), A*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWY</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0.01123023</v>
+      </c>
+      <c r="G29" t="n">
+        <v>54.132</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>(M=(0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24), A=(1, 2, 3, 4, 5, 6, 7, 8, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24)) | (M*=(), A*=(9,))</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>7.629e-05</v>
+      </c>
+      <c r="G30" t="n">
+        <v>97.35899999999999</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>(M=(), A=(3,)) | (M*=(0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24), A*=(1, 2, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>3.588e-05</v>
+      </c>
+      <c r="G31" t="n">
+        <v>101.177</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>(M=(), A=(5,)) | (M*=(1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23), A*=(1, 2, 3, 4, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>27</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>0.04356444</v>
+      </c>
+      <c r="G32" t="n">
+        <v>138.595</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>(M=(), A=(11,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24), A*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>28</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>0.01737872</v>
+      </c>
+      <c r="G33" t="n">
+        <v>131.42</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>(M=(), A=(18,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23), A*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 19, 20, 21, 22, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>29</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>0.008188010000000001</v>
+      </c>
+      <c r="G34" t="n">
+        <v>23.83</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>(M=(), A=(13,)) | (M*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24), A*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>30</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>0.06738436</v>
+      </c>
+      <c r="G35" t="n">
+        <v>20.426</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>(M=(), A=(18,)) | (M*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23), A*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 19, 20, 21, 22, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>31</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWY</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>1.764e-05</v>
+      </c>
+      <c r="G36" t="n">
+        <v>51.881</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>(M=(0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24), A=(1, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23)) | (M*=(), A*=(2,))</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>32</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>7.629e-05</v>
+      </c>
+      <c r="G37" t="n">
+        <v>93.922</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>(M=(), A=(3,)) | (M*=(0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24), A*=(1, 2, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>33</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>3.588e-05</v>
+      </c>
+      <c r="G38" t="n">
+        <v>99.081</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>(M=(), A=(5,)) | (M*=(1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23), A*=(1, 2, 3, 4, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWY</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>0.02388513</v>
+      </c>
+      <c r="G39" t="n">
+        <v>76.033</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>(M=(), A=(12,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24), A*=(0, 1, 3, 4, 6, 7, 9, 10, 13, 15, 16, 18, 19, 21, 22, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWY</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>0.01737872</v>
+      </c>
+      <c r="G40" t="n">
+        <v>223.462</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>(M=(), A=(18,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23), A*=(0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 19, 21, 22, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWY</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>0.008188010000000001</v>
+      </c>
+      <c r="G41" t="n">
+        <v>39.848</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>(M=(), A=(13,)) | (M*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24), A*=(0, 1, 3, 4, 6, 7, 9, 10, 12, 15, 16, 18, 19, 21, 22, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWY</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>0.06738436</v>
+      </c>
+      <c r="G42" t="n">
+        <v>43.442</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>(M=(), A=(18,)) | (M*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23), A*=(0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 19, 21, 22, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>0.02388513</v>
+      </c>
+      <c r="G43" t="n">
+        <v>41.319</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>(M=(), A=(12,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24), A*=(0, 2, 4, 6, 8, 10, 14, 16, 18, 20, 22, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>0.01737872</v>
+      </c>
+      <c r="G44" t="n">
+        <v>57.01</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>(M=(), A=(18,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23), A*=(0, 2, 4, 6, 8, 10, 12, 14, 16, 20, 22, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>0.16607529</v>
+      </c>
+      <c r="G45" t="n">
+        <v>33.571</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>(M=(), A=(8,)) | (M*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24), A*=(0, 2, 4, 6, 10, 12, 14, 16, 18, 20, 22, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>0.06738436</v>
+      </c>
+      <c r="G46" t="n">
+        <v>87.971</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>(M=(), A=(18,)) | (M*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23), A*=(0, 2, 4, 6, 8, 10, 12, 14, 16, 20, 22, 24))</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>48</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>0.04356444</v>
+      </c>
+      <c r="G47" t="n">
+        <v>53.409</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>(M=(), A=(11,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24), A*=(1, 3, 5, 7, 9, 13, 15, 17, 19, 21, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>49</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>0.11863324</v>
+      </c>
+      <c r="G48" t="n">
+        <v>178.098</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>(M=(), A=(19,)) | (M*=(0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23), A*=(1, 3, 5, 7, 9, 11, 13, 15, 17, 21, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>50</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1.11406493</v>
+      </c>
+      <c r="G49" t="n">
+        <v>240.151</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>(M=(2,), A=(13,)) | (M*=(1, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24), A*=(1, 3, 5, 7, 9, 11, 15, 17, 19, 21, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>51</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>0.00618219</v>
+      </c>
+      <c r="G50" t="n">
+        <v>13.406</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>(M=(), A=(19,)) | (M*=(1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23), A*=(1, 3, 5, 7, 9, 11, 13, 15, 17, 21, 23))</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>55</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ACDEFGHIJKLMNOPQRSTVX</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ACDEFGHIJKLMNOPQRSTVX</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>0.0022583</v>
+      </c>
+      <c r="G51" t="n">
+        <v>208.627</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>(M=(), A=(23,)) | (M*=(0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 21, 23), A*=(0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 21))</t>
         </is>
       </c>
     </row>
@@ -9784,984 +10854,984 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Estado inicial</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>10000000000000000000000000</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Sistema:</t>
         </is>
       </c>
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Sistema Candidato:</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D3" s="18" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>PRUEBAS  BIPARTICIONES</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>IBQNodos</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>#Prueba</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Alcance o Purview (t+1)</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Mecanismo(t)</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Partición</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Pérdida</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Tiempo</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n">
+      <c r="A6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D6" s="19" t="n"/>
-      <c r="E6" s="19" t="n"/>
-      <c r="F6" s="19" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="n">
+      <c r="A7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D7" s="20" t="n"/>
-      <c r="E7" s="20" t="n"/>
-      <c r="F7" s="20" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n">
+      <c r="A8" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D8" s="19" t="n"/>
-      <c r="E8" s="19" t="n"/>
-      <c r="F8" s="19" t="n"/>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="n">
+      <c r="A9" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="n"/>
-      <c r="F9" s="20" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n">
+      <c r="A10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="19" t="n"/>
-      <c r="F10" s="19" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="n">
+      <c r="A11" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D11" s="20" t="n"/>
-      <c r="E11" s="20" t="n"/>
-      <c r="F11" s="20" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="n">
+      <c r="A12" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C12" s="19" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="19" t="n"/>
+      <c r="D12" s="4" t="n"/>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n">
+      <c r="A13" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D13" s="19" t="n"/>
-      <c r="E13" s="19" t="n"/>
-      <c r="F13" s="19" t="n"/>
+      <c r="D13" s="4" t="n"/>
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="n">
+      <c r="A14" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D14" s="20" t="n"/>
-      <c r="E14" s="20" t="n"/>
-      <c r="F14" s="20" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n">
+      <c r="A15" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D15" s="19" t="n"/>
-      <c r="E15" s="19" t="n"/>
-      <c r="F15" s="19" t="n"/>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="n">
+      <c r="A16" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C16" s="20" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D16" s="20" t="n"/>
-      <c r="E16" s="20" t="n"/>
-      <c r="F16" s="20" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="n">
+      <c r="A17" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D17" s="19" t="n"/>
-      <c r="E17" s="19" t="n"/>
-      <c r="F17" s="19" t="n"/>
+      <c r="D17" s="4" t="n"/>
+      <c r="E17" s="4" t="n"/>
+      <c r="F17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="n">
+      <c r="A18" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C18" s="20" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="20" t="n"/>
-      <c r="F18" s="20" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="n">
+      <c r="A19" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="19" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C19" s="19" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D19" s="19" t="n"/>
-      <c r="E19" s="19" t="n"/>
-      <c r="F19" s="19" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="n">
+      <c r="A20" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="19" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C20" s="19" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D20" s="19" t="n"/>
-      <c r="E20" s="19" t="n"/>
-      <c r="F20" s="19" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="n">
+      <c r="A21" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C21" s="20" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D21" s="20" t="n"/>
-      <c r="E21" s="20" t="n"/>
-      <c r="F21" s="20" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="n">
+      <c r="A22" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B22" s="19" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C22" s="19" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D22" s="19" t="n"/>
-      <c r="E22" s="19" t="n"/>
-      <c r="F22" s="19" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="n">
+      <c r="A23" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C23" s="20" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D23" s="20" t="n"/>
-      <c r="E23" s="20" t="n"/>
-      <c r="F23" s="20" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="n">
+      <c r="A24" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B24" s="19" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C24" s="19" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D24" s="19" t="n"/>
-      <c r="E24" s="19" t="n"/>
-      <c r="F24" s="19" t="n"/>
+      <c r="D24" s="4" t="n"/>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="20" t="n">
+      <c r="A25" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="B25" s="20" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C25" s="20" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D25" s="20" t="n"/>
-      <c r="E25" s="20" t="n"/>
-      <c r="F25" s="20" t="n"/>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="n">
+      <c r="A26" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B26" s="19" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="C26" s="19" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D26" s="19" t="n"/>
-      <c r="E26" s="19" t="n"/>
-      <c r="F26" s="19" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="n">
+      <c r="A27" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="B27" s="19" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C27" s="19" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D27" s="19" t="n"/>
-      <c r="E27" s="19" t="n"/>
-      <c r="F27" s="19" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="20" t="n">
+      <c r="A28" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B28" s="20" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C28" s="20" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D28" s="20" t="n"/>
-      <c r="E28" s="20" t="n"/>
-      <c r="F28" s="20" t="n"/>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="n">
+      <c r="A29" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="B29" s="19" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C29" s="19" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D29" s="19" t="n"/>
-      <c r="E29" s="19" t="n"/>
-      <c r="F29" s="19" t="n"/>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="20" t="n">
+      <c r="A30" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="B30" s="20" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C30" s="20" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D30" s="20" t="n"/>
-      <c r="E30" s="20" t="n"/>
-      <c r="F30" s="20" t="n"/>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="n">
+      <c r="A31" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="B31" s="19" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C31" s="19" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D31" s="19" t="n"/>
-      <c r="E31" s="19" t="n"/>
-      <c r="F31" s="19" t="n"/>
+      <c r="D31" s="4" t="n"/>
+      <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="20" t="n">
+      <c r="A32" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="B32" s="20" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C32" s="20" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D32" s="20" t="n"/>
-      <c r="E32" s="20" t="n"/>
-      <c r="F32" s="20" t="n"/>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="19" t="n">
+      <c r="A33" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="B33" s="19" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="C33" s="19" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D33" s="19" t="n"/>
-      <c r="E33" s="19" t="n"/>
-      <c r="F33" s="19" t="n"/>
+      <c r="D33" s="4" t="n"/>
+      <c r="E33" s="4" t="n"/>
+      <c r="F33" s="4" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="19" t="n">
+      <c r="A34" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="B34" s="19" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="C34" s="19" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D34" s="19" t="n"/>
-      <c r="E34" s="19" t="n"/>
-      <c r="F34" s="19" t="n"/>
+      <c r="D34" s="4" t="n"/>
+      <c r="E34" s="4" t="n"/>
+      <c r="F34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="20" t="n">
+      <c r="A35" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="B35" s="20" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="C35" s="20" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D35" s="20" t="n"/>
-      <c r="E35" s="20" t="n"/>
-      <c r="F35" s="20" t="n"/>
+      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="5" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="19" t="n">
+      <c r="A36" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="B36" s="19" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="C36" s="19" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D36" s="19" t="n"/>
-      <c r="E36" s="19" t="n"/>
-      <c r="F36" s="19" t="n"/>
+      <c r="D36" s="4" t="n"/>
+      <c r="E36" s="4" t="n"/>
+      <c r="F36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="20" t="n">
+      <c r="A37" s="5" t="n">
         <v>32</v>
       </c>
-      <c r="B37" s="20" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="C37" s="20" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D37" s="20" t="n"/>
-      <c r="E37" s="20" t="n"/>
-      <c r="F37" s="20" t="n"/>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="5" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="19" t="n">
+      <c r="A38" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="B38" s="19" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="C38" s="19" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D38" s="19" t="n"/>
-      <c r="E38" s="19" t="n"/>
-      <c r="F38" s="19" t="n"/>
+      <c r="D38" s="4" t="n"/>
+      <c r="E38" s="4" t="n"/>
+      <c r="F38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="20" t="n">
+      <c r="A39" s="5" t="n">
         <v>34</v>
       </c>
-      <c r="B39" s="20" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="C39" s="20" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D39" s="20" t="n"/>
-      <c r="E39" s="20" t="n"/>
-      <c r="F39" s="20" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="19" t="n">
+      <c r="A40" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="B40" s="19" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="C40" s="19" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D40" s="19" t="n"/>
-      <c r="E40" s="19" t="n"/>
-      <c r="F40" s="19" t="n"/>
+      <c r="D40" s="4" t="n"/>
+      <c r="E40" s="4" t="n"/>
+      <c r="F40" s="4" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="19" t="n">
+      <c r="A41" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="B41" s="19" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="C41" s="19" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D41" s="19" t="n"/>
-      <c r="E41" s="19" t="n"/>
-      <c r="F41" s="19" t="n"/>
+      <c r="D41" s="4" t="n"/>
+      <c r="E41" s="4" t="n"/>
+      <c r="F41" s="4" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="20" t="n">
+      <c r="A42" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="B42" s="20" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="C42" s="20" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D42" s="20" t="n"/>
-      <c r="E42" s="20" t="n"/>
-      <c r="F42" s="20" t="n"/>
+      <c r="D42" s="5" t="n"/>
+      <c r="E42" s="5" t="n"/>
+      <c r="F42" s="5" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="19" t="n">
+      <c r="A43" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="B43" s="19" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="C43" s="19" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D43" s="19" t="n"/>
-      <c r="E43" s="19" t="n"/>
-      <c r="F43" s="19" t="n"/>
+      <c r="D43" s="4" t="n"/>
+      <c r="E43" s="4" t="n"/>
+      <c r="F43" s="4" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="20" t="n">
+      <c r="A44" s="5" t="n">
         <v>39</v>
       </c>
-      <c r="B44" s="20" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="C44" s="20" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D44" s="20" t="n"/>
-      <c r="E44" s="20" t="n"/>
-      <c r="F44" s="20" t="n"/>
+      <c r="D44" s="5" t="n"/>
+      <c r="E44" s="5" t="n"/>
+      <c r="F44" s="5" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="19" t="n">
+      <c r="A45" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="B45" s="19" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="C45" s="19" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D45" s="19" t="n"/>
-      <c r="E45" s="19" t="n"/>
-      <c r="F45" s="19" t="n"/>
+      <c r="D45" s="4" t="n"/>
+      <c r="E45" s="4" t="n"/>
+      <c r="F45" s="4" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="20" t="n">
+      <c r="A46" s="5" t="n">
         <v>41</v>
       </c>
-      <c r="B46" s="20" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="C46" s="20" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D46" s="20" t="n"/>
-      <c r="E46" s="20" t="n"/>
-      <c r="F46" s="20" t="n"/>
+      <c r="D46" s="5" t="n"/>
+      <c r="E46" s="5" t="n"/>
+      <c r="F46" s="5" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="19" t="n">
+      <c r="A47" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="B47" s="19" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="C47" s="19" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D47" s="19" t="n"/>
-      <c r="E47" s="19" t="n"/>
-      <c r="F47" s="19" t="n"/>
+      <c r="D47" s="4" t="n"/>
+      <c r="E47" s="4" t="n"/>
+      <c r="F47" s="4" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="19" t="n">
+      <c r="A48" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="B48" s="19" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="C48" s="19" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D48" s="19" t="n"/>
-      <c r="E48" s="19" t="n"/>
-      <c r="F48" s="19" t="n"/>
+      <c r="D48" s="4" t="n"/>
+      <c r="E48" s="4" t="n"/>
+      <c r="F48" s="4" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="20" t="n">
+      <c r="A49" s="5" t="n">
         <v>44</v>
       </c>
-      <c r="B49" s="20" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="C49" s="20" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D49" s="20" t="n"/>
-      <c r="E49" s="20" t="n"/>
-      <c r="F49" s="20" t="n"/>
+      <c r="D49" s="5" t="n"/>
+      <c r="E49" s="5" t="n"/>
+      <c r="F49" s="5" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="19" t="n">
+      <c r="A50" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="B50" s="19" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="C50" s="19" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D50" s="19" t="n"/>
-      <c r="E50" s="19" t="n"/>
-      <c r="F50" s="19" t="n"/>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="20" t="n">
+      <c r="A51" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="B51" s="20" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="C51" s="20" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D51" s="20" t="n"/>
-      <c r="E51" s="20" t="n"/>
-      <c r="F51" s="20" t="n"/>
+      <c r="D51" s="5" t="n"/>
+      <c r="E51" s="5" t="n"/>
+      <c r="F51" s="5" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="19" t="n">
+      <c r="A52" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="B52" s="19" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="C52" s="19" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D52" s="19" t="n"/>
-      <c r="E52" s="19" t="n"/>
-      <c r="F52" s="19" t="n"/>
+      <c r="D52" s="4" t="n"/>
+      <c r="E52" s="4" t="n"/>
+      <c r="F52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="20" t="n">
+      <c r="A53" s="5" t="n">
         <v>48</v>
       </c>
-      <c r="B53" s="20" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="C53" s="20" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D53" s="20" t="n"/>
-      <c r="E53" s="20" t="n"/>
-      <c r="F53" s="20" t="n"/>
+      <c r="D53" s="5" t="n"/>
+      <c r="E53" s="5" t="n"/>
+      <c r="F53" s="5" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="19" t="n">
+      <c r="A54" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="B54" s="19" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="C54" s="19" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D54" s="19" t="n"/>
-      <c r="E54" s="19" t="n"/>
-      <c r="F54" s="19" t="n"/>
+      <c r="D54" s="4" t="n"/>
+      <c r="E54" s="4" t="n"/>
+      <c r="F54" s="4" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="21" t="n">
+      <c r="A55" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="B55" s="22" t="inlineStr">
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>ACDEFGHIJKLMNOPQRSTVXZ</t>
         </is>
       </c>
-      <c r="C55" s="22" t="inlineStr">
+      <c r="C55" s="7" t="inlineStr">
         <is>
           <t>ACDEFGHIJKLMNOPQRSTVXZ</t>
         </is>
       </c>
-      <c r="D55" s="22" t="n"/>
-      <c r="E55" s="22" t="n"/>
-      <c r="F55" s="22" t="n"/>
+      <c r="D55" s="7" t="n"/>
+      <c r="E55" s="7" t="n"/>
+      <c r="F55" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Add Julia implementation for IBQNodos n=26 (memory-efficient via mmap)
</commit_message>
<xml_diff>
--- a/DatosIBQNodos2026.xlsx
+++ b/DatosIBQNodos2026.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plataforma" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10A-IBQNodos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15B-IBQNodos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20A-IBQNodos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22A-IBQNodos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25A-IBQNodos" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26A-Elementos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Plataforma" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="10A-IBQNodos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="15B-IBQNodos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="20A-IBQNodos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="22A-IBQNodos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="25A-IBQNodos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="26A-Elementos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="26A-IBQNodos" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1012,7 +1013,6 @@
   <mergeCells count="17">
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="B8:H8"/>
-    <mergeCell ref="A23:H23"/>
     <mergeCell ref="B26:H26"/>
     <mergeCell ref="B9:H9"/>
     <mergeCell ref="B27:H27"/>
@@ -1024,9 +1024,10 @@
     <mergeCell ref="B25:H25"/>
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A23:H23"/>
     <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B5:H5"/>
     <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B5:H5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11843,4 +11844,50 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>#Prueba</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Mecanismo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>IBQNodos_φ</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>IBQNodos_t(s)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Partición_IBQNodos</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
n=26 completado (50/50) + infraestructura n=27 lista
</commit_message>
<xml_diff>
--- a/DatosIBQNodos2026.xlsx
+++ b/DatosIBQNodos2026.xlsx
@@ -15,6 +15,9 @@
     <sheet name="25A-IBQNodos" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="26A-Elementos" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="26A-IBQNodos" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="26A-IBQNodos-Julia" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="27A-Elementos" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="27A-IBQNodos" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1014,8 +1017,8 @@
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="B8:H8"/>
     <mergeCell ref="B26:H26"/>
+    <mergeCell ref="B27:H27"/>
     <mergeCell ref="B9:H9"/>
-    <mergeCell ref="B27:H27"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="B12:H12"/>
     <mergeCell ref="B6:H6"/>
@@ -1029,6 +1032,907 @@
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="B11:H11"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Estado inicial</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>100000000000000000000000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sistema:</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Sistema Candidato:</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PRUEBAS  BIPARTICIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>IBQNodos</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>#Prueba</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Alcance o Purview (t+1)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Mecanismo(t)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Partición</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Pérdida</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Tiempo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>27</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>28</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>29</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>30</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>31</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>32</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>33</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>38</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUV</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUV</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>39</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>48</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>49</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>50</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>#Prueba</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Mecanismo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>φ (IBQNodos)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Tiempo(s)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Partición</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>(pendiente — correr main_ibqnodos27.jl)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10948,9 +11852,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0.09759676</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>255.364</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -10966,9 +11878,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0.24545497</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>381.714</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -10984,9 +11904,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0.25417846</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>272.884</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -11002,9 +11930,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0.14985549</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>379.052</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -11020,9 +11956,17 @@
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0.01644427</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>94.003</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
@@ -11038,9 +11982,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0.0003739</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>598.5940000000001</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -11056,9 +12008,17 @@
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0.00229689</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>590.463</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -11074,9 +12034,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0.09759676</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>49.707</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -11092,9 +12060,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>0.07539019</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>43.384</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -11110,9 +12086,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>0.25417846</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>73.82899999999999</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -11128,9 +12112,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>0.14985549</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>46.164</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -11146,9 +12138,17 @@
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0.01644427</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>70.53400000000001</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
@@ -11164,9 +12164,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>0.0003739</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>580.196</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -11182,9 +12190,17 @@
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>0.00229689</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>508.807</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -11200,9 +12216,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0.32270175</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>34.361</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
@@ -11218,9 +12242,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="n"/>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>0.07539019</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>43.984</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -11236,9 +12268,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0.29829895</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>41.795</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
@@ -11254,9 +12294,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>0.14985549</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>44.634</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -11272,9 +12320,17 @@
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="n"/>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>0.02085802</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>68.749</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
@@ -11290,9 +12346,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D25" s="5" t="n"/>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25" s="5" t="n"/>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>0.00312567</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>580.373</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -11308,9 +12372,17 @@
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>0.00229689</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>614.285</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -11326,9 +12398,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0.32270175</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>299.695</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
@@ -11344,9 +12424,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>0.07539019</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>375.791</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -11362,9 +12450,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>0.29829895</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>368.502</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
@@ -11380,9 +12476,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D30" s="5" t="n"/>
-      <c r="E30" s="5" t="n"/>
-      <c r="F30" s="5" t="n"/>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>0.14985549</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>354.067</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -11398,9 +12502,17 @@
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>0.02085802</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>335.748</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
@@ -11416,9 +12528,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D32" s="5" t="n"/>
-      <c r="E32" s="5" t="n"/>
-      <c r="F32" s="5" t="n"/>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>0.00312567</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>782.605</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -11434,9 +12554,17 @@
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D33" s="4" t="n"/>
-      <c r="E33" s="4" t="n"/>
-      <c r="F33" s="4" t="n"/>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>0.00229689</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>766.937</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -11452,9 +12580,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="4" t="n"/>
-      <c r="F34" s="4" t="n"/>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>0.09759676</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>399.421</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
@@ -11470,9 +12606,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D35" s="5" t="n"/>
-      <c r="E35" s="5" t="n"/>
-      <c r="F35" s="5" t="n"/>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>0.07539019</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>41.709</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -11488,9 +12632,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D36" s="4" t="n"/>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="4" t="n"/>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>0.25417846</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>42.764</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
@@ -11506,9 +12658,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D37" s="5" t="n"/>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37" s="5" t="n"/>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>0.14985549</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>37.79</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -11524,9 +12684,17 @@
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D38" s="4" t="n"/>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>0.01644427</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>94.925</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
@@ -11542,9 +12710,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D39" s="5" t="n"/>
-      <c r="E39" s="5" t="n"/>
-      <c r="F39" s="5" t="n"/>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>0.0003739</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>487.613</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -11560,9 +12736,17 @@
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D40" s="4" t="n"/>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="4" t="n"/>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[0, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>0.00229689</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>501.491</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -11578,9 +12762,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D41" s="4" t="n"/>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="n"/>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>0.09759676</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>100.934</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n">
@@ -11596,9 +12788,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D42" s="5" t="n"/>
-      <c r="E42" s="5" t="n"/>
-      <c r="F42" s="5" t="n"/>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>0.24545497</v>
+      </c>
+      <c r="F42" s="5" t="n">
+        <v>168.634</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -11614,9 +12814,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D43" s="4" t="n"/>
-      <c r="E43" s="4" t="n"/>
-      <c r="F43" s="4" t="n"/>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>0.25417846</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>162.737</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n">
@@ -11632,9 +12840,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D44" s="5" t="n"/>
-      <c r="E44" s="5" t="n"/>
-      <c r="F44" s="5" t="n"/>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="n">
+        <v>0.31220007</v>
+      </c>
+      <c r="F44" s="5" t="n">
+        <v>91.35299999999999</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -11650,9 +12866,17 @@
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D45" s="4" t="n"/>
-      <c r="E45" s="4" t="n"/>
-      <c r="F45" s="4" t="n"/>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>0.01644427</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>350.006</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n">
@@ -11668,9 +12892,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D46" s="5" t="n"/>
-      <c r="E46" s="5" t="n"/>
-      <c r="F46" s="5" t="n"/>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="n">
+        <v>0.0003739</v>
+      </c>
+      <c r="F46" s="5" t="n">
+        <v>517.148</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -11686,9 +12918,17 @@
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D47" s="4" t="n"/>
-      <c r="E47" s="4" t="n"/>
-      <c r="F47" s="4" t="n"/>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>0.00371623</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>443.732</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
@@ -11704,9 +12944,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D48" s="4" t="n"/>
-      <c r="E48" s="4" t="n"/>
-      <c r="F48" s="4" t="n"/>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>0.32270175</v>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>247.456</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n">
@@ -11722,9 +12970,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D49" s="5" t="n"/>
-      <c r="E49" s="5" t="n"/>
-      <c r="F49" s="5" t="n"/>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="n">
+        <v>0.07539019</v>
+      </c>
+      <c r="F49" s="5" t="n">
+        <v>161.78</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n">
@@ -11740,9 +12996,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
-      <c r="D50" s="4" t="n"/>
-      <c r="E50" s="4" t="n"/>
-      <c r="F50" s="4" t="n"/>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>0.29829895</v>
+      </c>
+      <c r="F50" s="4" t="n">
+        <v>191.057</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
@@ -11758,9 +13022,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
-      <c r="D51" s="5" t="n"/>
-      <c r="E51" s="5" t="n"/>
-      <c r="F51" s="5" t="n"/>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="n">
+        <v>0.14985549</v>
+      </c>
+      <c r="F51" s="5" t="n">
+        <v>107.919</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
@@ -11776,9 +13048,17 @@
           <t>ABDEGHJKMNPQSTVWYZ</t>
         </is>
       </c>
-      <c r="D52" s="4" t="n"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="4" t="n"/>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>0.02085802</v>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>349.727</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n">
@@ -11794,9 +13074,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
-      <c r="D53" s="5" t="n"/>
-      <c r="E53" s="5" t="n"/>
-      <c r="F53" s="5" t="n"/>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="n">
+        <v>0.00312567</v>
+      </c>
+      <c r="F53" s="5" t="n">
+        <v>410.066</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -11812,9 +13100,17 @@
           <t>BDFHJLNPRTVXZ</t>
         </is>
       </c>
-      <c r="D54" s="4" t="n"/>
-      <c r="E54" s="4" t="n"/>
-      <c r="F54" s="4" t="n"/>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>0.00229689</v>
+      </c>
+      <c r="F54" s="4" t="n">
+        <v>410.501</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n">
@@ -11830,9 +13126,17 @@
           <t>ACDEFGHIJKLMNOPQRSTVXZ</t>
         </is>
       </c>
-      <c r="D55" s="7" t="n"/>
-      <c r="E55" s="7" t="n"/>
-      <c r="F55" s="7" t="n"/>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 21, 23, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>0.00946754</v>
+      </c>
+      <c r="F55" s="7" t="n">
+        <v>20.236</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -11890,4 +13194,1350 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>#Prueba</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Mecanismo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>φ (IBQNodos)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Tiempo(s)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Partición</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.09759676</v>
+      </c>
+      <c r="E2" t="n">
+        <v>255.364</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.24545497</v>
+      </c>
+      <c r="E3" t="n">
+        <v>381.714</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.25417846</v>
+      </c>
+      <c r="E4" t="n">
+        <v>272.884</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.14985549</v>
+      </c>
+      <c r="E5" t="n">
+        <v>379.052</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.01644427</v>
+      </c>
+      <c r="E6" t="n">
+        <v>94.003</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.0003739</v>
+      </c>
+      <c r="E7" t="n">
+        <v>598.5940000000001</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.00229689</v>
+      </c>
+      <c r="E8" t="n">
+        <v>590.463</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.09759676</v>
+      </c>
+      <c r="E9" t="n">
+        <v>49.707</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.07539019</v>
+      </c>
+      <c r="E10" t="n">
+        <v>43.384</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.25417846</v>
+      </c>
+      <c r="E11" t="n">
+        <v>73.82899999999999</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.14985549</v>
+      </c>
+      <c r="E12" t="n">
+        <v>46.164</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.01644427</v>
+      </c>
+      <c r="E13" t="n">
+        <v>70.53400000000001</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0.0003739</v>
+      </c>
+      <c r="E14" t="n">
+        <v>580.196</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.00229689</v>
+      </c>
+      <c r="E15" t="n">
+        <v>508.807</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0.32270175</v>
+      </c>
+      <c r="E16" t="n">
+        <v>34.361</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.07539019</v>
+      </c>
+      <c r="E17" t="n">
+        <v>43.984</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0.29829895</v>
+      </c>
+      <c r="E18" t="n">
+        <v>41.795</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.14985549</v>
+      </c>
+      <c r="E19" t="n">
+        <v>44.634</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0.02085802</v>
+      </c>
+      <c r="E20" t="n">
+        <v>68.749</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0.00312567</v>
+      </c>
+      <c r="E21" t="n">
+        <v>580.373</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>0.00229689</v>
+      </c>
+      <c r="E22" t="n">
+        <v>614.285</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>0.32270175</v>
+      </c>
+      <c r="E23" t="n">
+        <v>299.695</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0.07539019</v>
+      </c>
+      <c r="E24" t="n">
+        <v>375.791</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>0.29829895</v>
+      </c>
+      <c r="E25" t="n">
+        <v>368.502</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0.14985549</v>
+      </c>
+      <c r="E26" t="n">
+        <v>354.067</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0.02085802</v>
+      </c>
+      <c r="E27" t="n">
+        <v>335.748</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0.00312567</v>
+      </c>
+      <c r="E28" t="n">
+        <v>782.605</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>0.00229689</v>
+      </c>
+      <c r="E29" t="n">
+        <v>766.937</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0.09759676</v>
+      </c>
+      <c r="E30" t="n">
+        <v>399.421</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0.07539019</v>
+      </c>
+      <c r="E31" t="n">
+        <v>41.709</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>0.25417846</v>
+      </c>
+      <c r="E32" t="n">
+        <v>42.764</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>0.14985549</v>
+      </c>
+      <c r="E33" t="n">
+        <v>37.79</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0.01644427</v>
+      </c>
+      <c r="E34" t="n">
+        <v>94.925</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0.0003739</v>
+      </c>
+      <c r="E35" t="n">
+        <v>487.613</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>0.00229689</v>
+      </c>
+      <c r="E36" t="n">
+        <v>501.491</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[0, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>0.09759676</v>
+      </c>
+      <c r="E37" t="n">
+        <v>100.934</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>0.24545497</v>
+      </c>
+      <c r="E38" t="n">
+        <v>168.634</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>0.25417846</v>
+      </c>
+      <c r="E39" t="n">
+        <v>162.737</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0.31220007</v>
+      </c>
+      <c r="E40" t="n">
+        <v>91.35299999999999</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>0.01644427</v>
+      </c>
+      <c r="E41" t="n">
+        <v>350.006</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>0.0003739</v>
+      </c>
+      <c r="E42" t="n">
+        <v>517.148</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>0.00371623</v>
+      </c>
+      <c r="E43" t="n">
+        <v>443.732</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>0.32270175</v>
+      </c>
+      <c r="E44" t="n">
+        <v>247.456</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>0.07539019</v>
+      </c>
+      <c r="E45" t="n">
+        <v>161.78</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0.29829895</v>
+      </c>
+      <c r="E46" t="n">
+        <v>191.057</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>0.14985549</v>
+      </c>
+      <c r="E47" t="n">
+        <v>107.919</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ABDEGHJKMNPQSTVWYZ</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>0.02085802</v>
+      </c>
+      <c r="E48" t="n">
+        <v>349.727</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 3, 4, 6, 7, 9, 10, 12, 13, 15, 16, 18, 19, 21, 22, 24, 25], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0.00312567</v>
+      </c>
+      <c r="E49" t="n">
+        <v>410.066</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVXZ</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>0.00229689</v>
+      </c>
+      <c r="E50" t="n">
+        <v>410.501</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ACDEFGHIJKLMNOPQRSTVXZ</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ACDEFGHIJKLMNOPQRSTVXZ</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>0.00946754</v>
+      </c>
+      <c r="E51" t="n">
+        <v>20.236</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 21, 23, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 21, 23, 25])</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: n=27 completado (50/50) — φ exacto, 5.1h total
</commit_message>
<xml_diff>
--- a/DatosIBQNodos2026.xlsx
+++ b/DatosIBQNodos2026.xlsx
@@ -18,6 +18,7 @@
     <sheet name="26A-IBQNodos-Julia" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="27A-Elementos" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="27A-IBQNodos" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="27A-IBQNodos-Julia" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1017,8 +1018,8 @@
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="B8:H8"/>
     <mergeCell ref="B26:H26"/>
+    <mergeCell ref="B9:H9"/>
     <mergeCell ref="B27:H27"/>
-    <mergeCell ref="B9:H9"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="B12:H12"/>
     <mergeCell ref="B6:H6"/>
@@ -1042,7 +1043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1139,6 +1140,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.00148478</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1071.102</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1154,6 +1166,17 @@
           <t>BDFHJLNPRTVX0</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.00062445</v>
+      </c>
+      <c r="F7" t="n">
+        <v>427.116</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1169,6 +1192,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.00169694</v>
+      </c>
+      <c r="F8" t="n">
+        <v>415.186</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1184,6 +1218,17 @@
           <t>BDFHJLNPRTVX0</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.00093043</v>
+      </c>
+      <c r="F9" t="n">
+        <v>422.556</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1199,6 +1244,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17])</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.00148478</v>
+      </c>
+      <c r="F10" t="n">
+        <v>431.661</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1214,6 +1270,17 @@
           <t>BDFHJLNPRTVX0</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18])</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0.00093043</v>
+      </c>
+      <c r="F11" t="n">
+        <v>426.875</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1229,6 +1296,17 @@
           <t>ABCDEFGHIJKLMNOPQR</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0.00176543</v>
+      </c>
+      <c r="F12" t="n">
+        <v>166.068</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1244,6 +1322,17 @@
           <t>BCDEFGHIJKLMNOPQRS</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0.00381273</v>
+      </c>
+      <c r="F13" t="n">
+        <v>168.143</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1259,6 +1348,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23])</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0.00148478</v>
+      </c>
+      <c r="F14" t="n">
+        <v>540.072</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1274,6 +1374,17 @@
           <t>BDFHJLNPRTVX0</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0.00093043</v>
+      </c>
+      <c r="F15" t="n">
+        <v>550.723</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1289,6 +1400,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0.00845945</v>
+      </c>
+      <c r="F16" t="n">
+        <v>221.709</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1304,6 +1426,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0.02811176</v>
+      </c>
+      <c r="F17" t="n">
+        <v>186.493</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1319,6 +1452,17 @@
           <t>BCDEFGHIJKLMNOPQRS</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17])</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>0.00381273</v>
+      </c>
+      <c r="F18" t="n">
+        <v>50.909</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1334,6 +1478,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0.00148478</v>
+      </c>
+      <c r="F19" t="n">
+        <v>932.557</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1349,6 +1504,17 @@
           <t>BDFHJLNPRTVX0</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0.00093043</v>
+      </c>
+      <c r="F20" t="n">
+        <v>953.232</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1364,6 +1530,17 @@
           <t>BDFHJLNPRTVX0</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0.00062445</v>
+      </c>
+      <c r="F21" t="n">
+        <v>953.645</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1379,6 +1556,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0.00169694</v>
+      </c>
+      <c r="F22" t="n">
+        <v>940.544</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1394,6 +1582,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0.02048361</v>
+      </c>
+      <c r="F23" t="n">
+        <v>179.851</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1409,6 +1608,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0.23788762</v>
+      </c>
+      <c r="F24" t="n">
+        <v>216.048</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1424,6 +1634,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0.01307973</v>
+      </c>
+      <c r="F25" t="n">
+        <v>178.963</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1439,6 +1660,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.08641857</v>
+      </c>
+      <c r="F26" t="n">
+        <v>180.258</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1454,6 +1686,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0.00148478</v>
+      </c>
+      <c r="F27" t="n">
+        <v>671.737</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1469,6 +1712,17 @@
           <t>BDFHJLNPRTVX0</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26])</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0.00093043</v>
+      </c>
+      <c r="F28" t="n">
+        <v>683.893</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1484,6 +1738,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0.21432137</v>
+      </c>
+      <c r="F29" t="n">
+        <v>212.97</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1499,6 +1764,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>0.15964895</v>
+      </c>
+      <c r="F30" t="n">
+        <v>215.95</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1514,6 +1790,17 @@
           <t>ACEGIKMOQSUWY</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26])</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0.00148478</v>
+      </c>
+      <c r="F31" t="n">
+        <v>818.888</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1529,6 +1816,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>0.32275659</v>
+      </c>
+      <c r="F32" t="n">
+        <v>154.632</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1544,6 +1842,17 @@
           <t>BCDEFGHIJKLMNOPQRS</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23])</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>0.00381273</v>
+      </c>
+      <c r="F33" t="n">
+        <v>285.782</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1559,6 +1868,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17])</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0.02811176</v>
+      </c>
+      <c r="F34" t="n">
+        <v>54.504</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1574,6 +1894,17 @@
           <t>ABCDEFGHIJKLMNOPQR</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0.00176543</v>
+      </c>
+      <c r="F35" t="n">
+        <v>109.925</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1589,6 +1920,17 @@
           <t>BCDEFGHIJKLMNOPQRS</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0.00381273</v>
+      </c>
+      <c r="F36" t="n">
+        <v>102.843</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1604,6 +1946,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17])</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0.01307973</v>
+      </c>
+      <c r="F37" t="n">
+        <v>47.826</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1619,6 +1972,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18])</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0.08641857</v>
+      </c>
+      <c r="F38" t="n">
+        <v>49.509</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1634,6 +1998,17 @@
           <t>ABCDEFGHIJKLMNOPQR</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0.00176543</v>
+      </c>
+      <c r="F39" t="n">
+        <v>161.607</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1649,6 +2024,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18])</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>0.15964895</v>
+      </c>
+      <c r="F40" t="n">
+        <v>45.482</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1664,6 +2050,17 @@
           <t>ABCDEFGHIJKLMNOPQR</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26])</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0.00176543</v>
+      </c>
+      <c r="F41" t="n">
+        <v>420.642</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1679,6 +2076,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17])</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>0.32275659</v>
+      </c>
+      <c r="F42" t="n">
+        <v>540.115</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1694,6 +2102,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUV</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21])</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>0.02208883</v>
+      </c>
+      <c r="F43" t="n">
+        <v>26.148</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1709,6 +2128,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23])</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>0.02811176</v>
+      </c>
+      <c r="F44" t="n">
+        <v>284.871</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1724,6 +2154,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>0.00845945</v>
+      </c>
+      <c r="F45" t="n">
+        <v>69.61499999999999</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1739,6 +2180,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>0.23788762</v>
+      </c>
+      <c r="F46" t="n">
+        <v>629.7910000000001</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1754,6 +2206,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0.02811176</v>
+      </c>
+      <c r="F47" t="n">
+        <v>583.885</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1769,6 +2232,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23])</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0.04399875</v>
+      </c>
+      <c r="F48" t="n">
+        <v>500.323</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1784,6 +2258,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0.01307973</v>
+      </c>
+      <c r="F49" t="n">
+        <v>61.001</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1799,6 +2284,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>0.08641857</v>
+      </c>
+      <c r="F50" t="n">
+        <v>66.345</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1814,6 +2310,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>0.01307973</v>
+      </c>
+      <c r="F51" t="n">
+        <v>473.832</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1829,6 +2336,17 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>0.04399875</v>
+      </c>
+      <c r="F52" t="n">
+        <v>61.318</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1844,6 +2362,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26])</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>0.02048361</v>
+      </c>
+      <c r="F53" t="n">
+        <v>932.629</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1859,6 +2388,17 @@
           <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0.04538554</v>
+      </c>
+      <c r="F54" t="n">
+        <v>59.09</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1874,11 +2414,18 @@
           <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
         </is>
       </c>
-    </row>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>0.04399875</v>
+      </c>
+      <c r="F55" t="n">
+        <v>436.337</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1929,6 +2476,1352 @@
       <c r="A2" t="inlineStr">
         <is>
           <t>(pendiente — correr main_ibqnodos27.jl)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>#Prueba</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Mecanismo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>φ (IBQNodos)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Tiempo(s)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Partición</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.00148478</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1071.102</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.00062445</v>
+      </c>
+      <c r="E3" t="n">
+        <v>427.116</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.00169694</v>
+      </c>
+      <c r="E4" t="n">
+        <v>415.186</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.00093043</v>
+      </c>
+      <c r="E5" t="n">
+        <v>422.556</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.00148478</v>
+      </c>
+      <c r="E6" t="n">
+        <v>431.661</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17])</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.00093043</v>
+      </c>
+      <c r="E7" t="n">
+        <v>426.875</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18])</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.00176543</v>
+      </c>
+      <c r="E8" t="n">
+        <v>166.068</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.00381273</v>
+      </c>
+      <c r="E9" t="n">
+        <v>168.143</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.00148478</v>
+      </c>
+      <c r="E10" t="n">
+        <v>540.072</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23])</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.00093043</v>
+      </c>
+      <c r="E11" t="n">
+        <v>550.723</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.00845945</v>
+      </c>
+      <c r="E12" t="n">
+        <v>221.709</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.02811176</v>
+      </c>
+      <c r="E13" t="n">
+        <v>186.493</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0.00381273</v>
+      </c>
+      <c r="E14" t="n">
+        <v>50.909</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17])</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.00148478</v>
+      </c>
+      <c r="E15" t="n">
+        <v>932.557</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0.00093043</v>
+      </c>
+      <c r="E16" t="n">
+        <v>953.232</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.00062445</v>
+      </c>
+      <c r="E17" t="n">
+        <v>953.645</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0.00169694</v>
+      </c>
+      <c r="E18" t="n">
+        <v>940.544</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.02048361</v>
+      </c>
+      <c r="E19" t="n">
+        <v>179.851</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0.23788762</v>
+      </c>
+      <c r="E20" t="n">
+        <v>216.048</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0.01307973</v>
+      </c>
+      <c r="E21" t="n">
+        <v>178.963</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>0.08641857</v>
+      </c>
+      <c r="E22" t="n">
+        <v>180.258</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>0.00148478</v>
+      </c>
+      <c r="E23" t="n">
+        <v>671.737</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0.00093043</v>
+      </c>
+      <c r="E24" t="n">
+        <v>683.893</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26])</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>0.21432137</v>
+      </c>
+      <c r="E25" t="n">
+        <v>212.97</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BDFHJLNPRTVX0</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0.15964895</v>
+      </c>
+      <c r="E26" t="n">
+        <v>215.95</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[3, 5, 7, 9, 11, 13, 15, 17, 19, 21, 23, 26])</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0.00148478</v>
+      </c>
+      <c r="E27" t="n">
+        <v>818.888</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26])</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ACEGIKMOQSUWY</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0.32275659</v>
+      </c>
+      <c r="E28" t="n">
+        <v>154.632</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[2, 4, 6, 8, 10, 12, 14, 16, 18, 20, 22, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>0.00381273</v>
+      </c>
+      <c r="E29" t="n">
+        <v>285.782</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23])</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0.02811176</v>
+      </c>
+      <c r="E30" t="n">
+        <v>54.504</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17])</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0.00176543</v>
+      </c>
+      <c r="E31" t="n">
+        <v>109.925</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>0.00381273</v>
+      </c>
+      <c r="E32" t="n">
+        <v>102.843</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>0.01307973</v>
+      </c>
+      <c r="E33" t="n">
+        <v>47.826</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17])</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0.08641857</v>
+      </c>
+      <c r="E34" t="n">
+        <v>49.509</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18])</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0.00176543</v>
+      </c>
+      <c r="E35" t="n">
+        <v>161.607</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>0.15964895</v>
+      </c>
+      <c r="E36" t="n">
+        <v>45.482</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18])</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>0.00176543</v>
+      </c>
+      <c r="E37" t="n">
+        <v>420.642</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26])</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>0.32275659</v>
+      </c>
+      <c r="E38" t="n">
+        <v>540.115</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17])</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUV</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUV</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>0.02208883</v>
+      </c>
+      <c r="E39" t="n">
+        <v>26.148</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21])</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0.02811176</v>
+      </c>
+      <c r="E40" t="n">
+        <v>284.871</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23])</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>0.00845945</v>
+      </c>
+      <c r="E41" t="n">
+        <v>69.61499999999999</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>0.23788762</v>
+      </c>
+      <c r="E42" t="n">
+        <v>629.7910000000001</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>0.02811176</v>
+      </c>
+      <c r="E43" t="n">
+        <v>583.885</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[0, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>0.04399875</v>
+      </c>
+      <c r="E44" t="n">
+        <v>500.323</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23])</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>0.01307973</v>
+      </c>
+      <c r="E45" t="n">
+        <v>61.001</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0.08641857</v>
+      </c>
+      <c r="E46" t="n">
+        <v>66.345</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>0.01307973</v>
+      </c>
+      <c r="E47" t="n">
+        <v>473.832</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>0.04399875</v>
+      </c>
+      <c r="E48" t="n">
+        <v>61.318</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24])</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0.02048361</v>
+      </c>
+      <c r="E49" t="n">
+        <v>932.629</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26])</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>0.04538554</v>
+      </c>
+      <c r="E50" t="n">
+        <v>59.09</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[1]) / (M=[0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>BCDEFGHIJKLMNOPQRSTUVWXYZ0</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>0.04399875</v>
+      </c>
+      <c r="E51" t="n">
+        <v>436.337</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>(M=Int64[], A=[0]) / (M=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26], A=[1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25])</t>
         </is>
       </c>
     </row>

</xml_diff>